<commit_message>
agrego implementacion modulo 4 tp3 (no finalizado, sin probar)
</commit_message>
<xml_diff>
--- a/server3/informe_donaciones.xlsx
+++ b/server3/informe_donaciones.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
   <si>
     <t>Categoría</t>
   </si>
@@ -33,6 +33,63 @@
   </si>
   <si>
     <t>Usuario Modificación</t>
+  </si>
+  <si>
+    <t>ROPA</t>
+  </si>
+  <si>
+    <t>Remeras</t>
+  </si>
+  <si>
+    <t>2025-10-26T20:10:38.208815</t>
+  </si>
+  <si>
+    <t>testuser</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Camperas</t>
+  </si>
+  <si>
+    <t>2025-10-26T20:10:47.323520</t>
+  </si>
+  <si>
+    <t>ALIMENTOS</t>
+  </si>
+  <si>
+    <t>Arroz</t>
+  </si>
+  <si>
+    <t>2025-10-26T20:10:54.931483</t>
+  </si>
+  <si>
+    <t>JUGUETES</t>
+  </si>
+  <si>
+    <t>Autitos</t>
+  </si>
+  <si>
+    <t>2025-10-26T20:11:02.073768</t>
+  </si>
+  <si>
+    <t>UTILES_ESCOLARES</t>
+  </si>
+  <si>
+    <t>Lapiz</t>
+  </si>
+  <si>
+    <t>2025-10-26T20:11:08.919104</t>
+  </si>
+  <si>
+    <t>2025-10-26T20:11:22.924053</t>
+  </si>
+  <si>
+    <t>Cuadernos</t>
+  </si>
+  <si>
+    <t>2025-10-26T20:11:47.284651</t>
   </si>
 </sst>
 </file>
@@ -77,14 +134,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="8.625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="16.4765625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="10.2734375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="8.09765625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="8.88671875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="9.28125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="24.65234375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="10.77734375" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="17.9921875" customWidth="true" bestFit="true"/>
   </cols>
@@ -112,6 +169,167 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="D2" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C3" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="D3" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="C4" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="D4" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C5" t="n" s="0">
+        <v>30.0</v>
+      </c>
+      <c r="D5" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C6" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="D6" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C7" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="D7" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C8" t="n" s="0">
+        <v>30.0</v>
+      </c>
+      <c r="D8" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>